<commit_message>
Programación multimedia Act1 y temario de SGE y desarrollo de interfaces
</commit_message>
<xml_diff>
--- a/Programación Multimedia/Tema1/Actividades/Actividad1.xlsx
+++ b/Programación Multimedia/Tema1/Actividades/Actividad1.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Android</t>
   </si>
@@ -39,13 +39,43 @@
     <t xml:space="preserve">Lenguaje base de desarrollo</t>
   </si>
   <si>
-    <t xml:space="preserve">actualmente kotlin</t>
+    <t xml:space="preserve">Kotlin/Java y C/C++</t>
+  </si>
+  <si>
+    <t>Swift</t>
+  </si>
+  <si>
+    <t>C++</t>
   </si>
   <si>
     <t xml:space="preserve">Modelo Principal de interfaz usuario</t>
   </si>
   <si>
+    <t xml:space="preserve">Material Design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UIKit, FundationFramework y cocoatouch</t>
+  </si>
+  <si>
+    <t>S60</t>
+  </si>
+  <si>
+    <t>wayland</t>
+  </si>
+  <si>
     <t xml:space="preserve">Caracterítica técnica aportada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ser opensource</t>
+  </si>
+  <si>
+    <t xml:space="preserve">combinación casi perfecta hard&amp;soft y pantalla multitáctil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multitarea, conectividad por paquetes de datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestos según esquinas</t>
   </si>
 </sst>
 </file>
@@ -95,11 +125,8 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -608,64 +635,86 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="2" max="8" width="11.57421875"/>
+    <col customWidth="1" min="2" max="3" width="11.57421875"/>
+    <col bestFit="1" customWidth="1" min="4" max="4" width="20.51171875"/>
+    <col customWidth="1" min="5" max="8" width="11.57421875"/>
   </cols>
   <sheetData>
     <row r="2" ht="35.25" customHeight="1">
       <c r="B2" s="1"/>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" ht="51" customHeight="1">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
     </row>
     <row r="4" ht="62.25" customHeight="1">
-      <c r="B4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="3" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="5" ht="51" customHeight="1">
-      <c r="B5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
+    <row r="5" ht="81" customHeight="1">
+      <c r="B5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="3" t="s">
+        <v>19</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>